<commit_message>
Adding pipeline for coregistration.
</commit_message>
<xml_diff>
--- a/Animals_Clearance_Turner_complete_list.xlsx
+++ b/Animals_Clearance_Turner_complete_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rja20/Documents/MATLAB/Bruker_radial_recon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D561B20C-6067-F14B-AC78-C54A5F0E98C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F470FEC-3A97-AA48-ADCA-BC36265BD60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4760" yWindow="2100" windowWidth="39980" windowHeight="26700" xr2:uid="{84E1B740-0BA9-6B4F-AA6B-2F5191EC9593}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$N$1:$N$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$L$1:$M$59</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$T$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Sheet2!$A$1:$B$18</definedName>
   </definedNames>
@@ -3967,7 +3967,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="N1:N58" xr:uid="{FFA5DD44-FC73-C044-A196-AFED27C59F6D}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="60" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>